<commit_message>
Advance Scheme Saathi to production-grade portal
- Security: Add Author Desk PIN gate (PIN: 1234) with session management and Lock capability
- Analytics: Implement live KPI stats endpoint (/api/admin/stats) and dashboard summary cards
- UX: Open SchemeFinder directly to citizens without forced login barrier
- Mobile: Add fixed mobile bottom navigation bar with active indicators and safe area padding
- PWA: Add web manifest (manifest.json) and mobile web app meta tags in index.html
- Schemes: Add real-time search filter and Check Eligibility / Ask AI action buttons on ExploreSchemes cards
- Design: Add institutional government scheme metrics bar to LandingPage
- Stepper: Fix z-index stacking on Track Application desktop progress connector line
- Backend: Clean CORS regex in main.py, auto-clear stale action_required on stage advance, and add full_name migration in database.py
</commit_message>
<xml_diff>
--- a/Admin_Data/User_Applications.xlsx
+++ b/Admin_Data/User_Applications.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Applications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1118,15 +1118,15 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2. Document Verification</t>
+          <t>3. SCA / Partner Review</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Under Document Verification</t>
+          <t>SCA / Channel Partner Review</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Your digital KYC and Caste certificate have been verified. Field verification by the district officer is scheduled between 05 Sep and 08 Sep 2026.</t>
+          <t>Test advance from API test</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-09-04 18:04:28</t>
+          <t>2026-09-12 16:17:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Track Application: AI-assisted application journey on mobile lookup, fix 401 on my-applications, and eliminate 404 console errors
</commit_message>
<xml_diff>
--- a/Admin_Data/User_Applications.xlsx
+++ b/Admin_Data/User_Applications.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -543,50 +543,50 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SS-2026-TL-6841</t>
+          <t>SS-2026-MFS-86C2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Citizen 1727</t>
+          <t>Applicant 9856</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9151541727</t>
+          <t>9645679856</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Term Loan</t>
+          <t>Micro Finance Scheme (MFS)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>₹ 150,000</t>
+          <t>₹ 1,40,000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Income Generating Activity</t>
+          <t>Micro Enterprise &amp; Retail Trade</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1. Application Submitted</t>
+          <t>2. Document Verification</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Application Submitted - Under Scrutiny</t>
+          <t>Under Document Verification</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -596,22 +596,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Application registered for mobile #9151541727. Awaiting Scrutiny Cell review.</t>
+          <t>Official Verification Note: Aadhaar e-KYC and digital category verification validated for Applicant 9856. Scrutiny in progress at New Delhi District Verification Cell.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -621,49 +621,49 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-06 04:19:18</t>
+          <t>2026-09-17 15:45:02</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-09-06 04:19:18</t>
+          <t>2026-09-17 15:45:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-5844</t>
+          <t>SS-2026-TL-6841</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sunita Devi</t>
+          <t>Citizen 1727</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9888615763</t>
+          <t>9151541727</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MFS</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Micro Finance Scheme (MFS)</t>
+          <t>Term Loan</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Rs 1,25,000</t>
+          <t>₹ 150,000</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dairy Farming and Cattle Feed</t>
+          <t>Income Generating Activity</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -686,22 +686,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-5844. Initial document verification in progress.</t>
+          <t>Application registered for mobile #9151541727. Awaiting Scrutiny Cell review.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -711,29 +711,29 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-05 13:42:47</t>
+          <t>2026-09-06 04:19:18</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-09-05 13:42:47</t>
+          <t>2026-09-06 04:19:18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-5626</t>
+          <t>SS-2026-MFS-5844</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Test User</t>
+          <t>Sunita Devi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8765676029</t>
+          <t>9888615763</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -743,30 +743,30 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Micro Finance Scheme</t>
+          <t>Micro Finance Scheme (MFS)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>₹ 1,50,000</t>
+          <t>Rs 1,25,000</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Retail Kirana Shop</t>
+          <t>Dairy Farming and Cattle Feed</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2. Document Verification</t>
+          <t>1. Application Submitted</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Under Document Verification</t>
+          <t>Application Submitted - Under Scrutiny</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -786,34 +786,34 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Author verified initial submission. Document verification in progress at District Scrutiny Cell.</t>
+          <t>Application registered successfully under #SS-2026-MFS-5844. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Keep your original Aadhaar and Caste certificates ready for verification visit.</t>
+          <t>None</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-04 18:09:10</t>
+          <t>2026-09-05 13:42:47</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-09-05 12:35:31</t>
+          <t>2026-09-05 13:42:47</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-2153</t>
+          <t>SS-2026-MFS-5626</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -848,15 +848,15 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1. Application Submitted</t>
+          <t>2. Document Verification</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Application Submitted - Under Scrutiny</t>
+          <t>Under Document Verification</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -881,29 +881,29 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-2153. Initial document verification in progress.</t>
+          <t>Author verified initial submission. Document verification in progress at District Scrutiny Cell.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Keep your original Aadhaar and Caste certificates ready for verification visit.</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:53</t>
+          <t>2026-09-04 18:09:10</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:53</t>
+          <t>2026-09-05 12:35:31</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-7582</t>
+          <t>SS-2026-MFS-2153</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-7582. Initial document verification in progress.</t>
+          <t>Application registered successfully under #SS-2026-MFS-2153. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -981,19 +981,19 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:45</t>
+          <t>2026-09-04 18:05:53</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:45</t>
+          <t>2026-09-04 18:05:53</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-1285</t>
+          <t>SS-2026-MFS-7582</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-1285. Initial document verification in progress.</t>
+          <t>Application registered successfully under #SS-2026-MFS-7582. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1071,29 +1071,29 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:36</t>
+          <t>2026-09-04 18:05:45</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:36</t>
+          <t>2026-09-04 18:05:45</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-8492</t>
+          <t>SS-2026-MFS-1285</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ramesh Chandra</t>
+          <t>Test User</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>XXXXXX4219</t>
+          <t>8765676029</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1103,30 +1103,30 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Micro Finance Scheme (MFS)</t>
+          <t>Micro Finance Scheme</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Rs 1,40,000</t>
+          <t>₹ 1,50,000</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Small Retail Kirana Store Expansion</t>
+          <t>Retail Kirana Shop</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3. SCA / Partner Review</t>
+          <t>1. Application Submitted</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>SCA / Channel Partner Review</t>
+          <t>Application Submitted - Under Scrutiny</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1136,22 +1136,22 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Test advance from API test</t>
+          <t>Application registered successfully under #SS-2026-MFS-1285. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1161,92 +1161,92 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-09-04 18:04:28</t>
+          <t>2026-09-04 18:05:36</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-09-12 16:17:31</t>
+          <t>2026-09-04 18:05:36</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SS-2026-ELS-3104</t>
+          <t>SS-2026-MFS-8492</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pooja Kumari</t>
+          <t>Ramesh Chandra</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>XXXXXX8832</t>
+          <t>XXXXXX4219</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ELS</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Educational Loan Scheme (ELS)</t>
+          <t>Micro Finance Scheme (MFS)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Rs 7,50,000</t>
+          <t>Rs 1,40,000</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>B.Tech Computer Science &amp; Engineering (4-Year Degree)</t>
+          <t>Small Retail Kirana Store Expansion</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>4. Bank Sanction</t>
+          <t>3. SCA / Partner Review</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Loan Sanctioned - Ready for Disbursement</t>
+          <t>SCA / Channel Partner Review</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Sanction letter #ELS-2026-9812 has been issued. Subsidized interest rate at 4.0% p.a. approved for the study tenure.</t>
+          <t>Test advance from API test</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Please visit the branch by 06 Sep 2026 with your admission letter original and bank passbook to sign the subsidy agreement.</t>
+          <t>None</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1256,95 +1256,185 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2026-09-04 18:04:28</t>
+          <t>2026-09-12 16:17:31</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>SS-2026-ELS-3104</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pooja Kumari</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>XXXXXX8832</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ELS</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Educational Loan Scheme (ELS)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Rs 7,50,000</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>B.Tech Computer Science &amp; Engineering (4-Year Degree)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4. Bank Sanction</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Loan Sanctioned - Ready for Disbursement</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Sanction letter #ELS-2026-9812 has been issued. Subsidized interest rate at 4.0% p.a. approved for the study tenure.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Please visit the branch by 06 Sep 2026 with your admission letter original and bank passbook to sign the subsidy agreement.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-09-04 18:04:28</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-09-04 18:04:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>SS-2026-TL-5521</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Manoj Meghwal</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>XXXXXX1904</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>TERM_LOAN</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Term Loan (TL)</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Rs 12,00,000</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Food Processing &amp; Packaging Unit</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>2. Document Verification</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Action Required - Document Clarification</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>ACTION_REQUIRED</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Scrutiny committee found that the annual income certificate submitted was issued in 2024. As per NSFDC policy, income certificate must be valid within the past 12 months.</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Please provide an updated Family Income Certificate for FY 2026-27 issued by Tehsildar. The current document uploaded has expired.</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>2026-09-04 18:04:28</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>2026-09-04 18:04:28</t>
         </is>

</xml_diff>

<commit_message>
Implement end-to-end 5-stage application & document lifecycle with completeness gatekeeper
</commit_message>
<xml_diff>
--- a/Admin_Data/User_Applications.xlsx
+++ b/Admin_Data/User_Applications.xlsx
@@ -1208,20 +1208,20 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3. SCA / Partner Review</t>
+          <t>5. Disbursement (DBT)</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>SCA / Channel Partner Review</t>
+          <t>Disbursed - Loan Credited</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DISBURSED</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Test advance from API test</t>
+          <t>DBT Disbursement completed! Concessional loan of ₹ 1,75,000 credited. Ref UTR: UTR9876543210.</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2026-09-12 16:17:31</t>
+          <t>2026-09-17 16:21:14</t>
         </is>
       </c>
     </row>

</xml_diff>